<commit_message>
GMFCL & GMFCR NF
</commit_message>
<xml_diff>
--- a/src/data/TestData.xlsx
+++ b/src/data/TestData.xlsx
@@ -5,10 +5,10 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bcharles\source\Repository\CDBatch_Migration\mar13\RC-Batch-Partial-Regression\src\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bcharles\source\Repository\CDBatch_Migration\Mar16\RC-Batch-Partial-Regression\src\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2367EBFB-4578-4843-B4A0-4292D5FEED91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2975CC4F-A7FC-4CAB-AF14-73DFF113FB1D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="85">
   <si>
     <t>ScenarioId</t>
   </si>
@@ -248,6 +248,36 @@
   </si>
   <si>
     <t>BNS_Comm_Lookup.xml</t>
+  </si>
+  <si>
+    <t>GMF</t>
+  </si>
+  <si>
+    <t>GMFCL</t>
+  </si>
+  <si>
+    <t>GMF_CL</t>
+  </si>
+  <si>
+    <t>GMFCL_HappyPath.XIF</t>
+  </si>
+  <si>
+    <t>GMF_ReturnFile</t>
+  </si>
+  <si>
+    <t>GMFCL_NFHappyPath</t>
+  </si>
+  <si>
+    <t>GMFCR</t>
+  </si>
+  <si>
+    <t>GMF_CR</t>
+  </si>
+  <si>
+    <t>GMFCR_HappyPath.XIF</t>
+  </si>
+  <si>
+    <t>GMFCR_NFHappyPath</t>
   </si>
 </sst>
 </file>
@@ -289,7 +319,28 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="2">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -624,7 +675,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:P19"/>
+  <dimension ref="A1:P21"/>
   <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="43.69921875" bestFit="1" customWidth="1"/>
@@ -1128,7 +1179,59 @@
         <v>30</v>
       </c>
     </row>
+    <row r="20" spans="1:7" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>80</v>
+      </c>
+      <c r="B20" t="s">
+        <v>75</v>
+      </c>
+      <c r="C20" t="s">
+        <v>76</v>
+      </c>
+      <c r="D20" t="s">
+        <v>77</v>
+      </c>
+      <c r="E20" t="s">
+        <v>78</v>
+      </c>
+      <c r="F20" t="s">
+        <v>20</v>
+      </c>
+      <c r="G20" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>84</v>
+      </c>
+      <c r="B21" t="s">
+        <v>75</v>
+      </c>
+      <c r="C21" t="s">
+        <v>81</v>
+      </c>
+      <c r="D21" t="s">
+        <v>82</v>
+      </c>
+      <c r="E21" t="s">
+        <v>83</v>
+      </c>
+      <c r="F21" t="s">
+        <v>20</v>
+      </c>
+      <c r="G21" t="s">
+        <v>79</v>
+      </c>
+    </row>
   </sheetData>
+  <conditionalFormatting sqref="A20">
+    <cfRule type="duplicateValues" dxfId="1" priority="2"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A21">
+    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
     <ignoredError sqref="A1:P15 B16:P16" numberStoredAsText="1"/>

</xml_diff>

<commit_message>
BNS_COMM Invalid Batch Number
</commit_message>
<xml_diff>
--- a/src/data/TestData.xlsx
+++ b/src/data/TestData.xlsx
@@ -5,10 +5,10 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bcharles\source\Repository\CDBatch_Migration\Mar_17\RC-Batch-Partial-Regression\src\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bcharles\source\Repository\CDBatch_Migration\Mar18\RC_Batch_Full_Regression\src\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C44AC38C-2E9D-42B7-A781-F2B4674BFBFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{865E4784-ED08-4307-89E4-40C0F97318D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="208" uniqueCount="91">
   <si>
     <t>ScenarioId</t>
   </si>
@@ -287,6 +287,15 @@
   </si>
   <si>
     <t>BNS_COMM_Amendment</t>
+  </si>
+  <si>
+    <t>BNS_COMM_NF_Duplicate_BatchNumber</t>
+  </si>
+  <si>
+    <t>BNS_COMM_Renewal_Duplicate_BatchNumber</t>
+  </si>
+  <si>
+    <t>BNS_COMM_Discharge_Duplicate_BatchNumber</t>
   </si>
 </sst>
 </file>
@@ -684,7 +693,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:P23"/>
+  <dimension ref="A1:P26"/>
   <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="43.69921875" bestFit="1" customWidth="1"/>
@@ -1286,6 +1295,87 @@
         <v>30</v>
       </c>
     </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>88</v>
+      </c>
+      <c r="B24" t="s">
+        <v>27</v>
+      </c>
+      <c r="C24" t="s">
+        <v>27</v>
+      </c>
+      <c r="D24" t="s">
+        <v>28</v>
+      </c>
+      <c r="E24" t="s">
+        <v>29</v>
+      </c>
+      <c r="F24" t="s">
+        <v>20</v>
+      </c>
+      <c r="G24" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>89</v>
+      </c>
+      <c r="B25" t="s">
+        <v>27</v>
+      </c>
+      <c r="C25" t="s">
+        <v>27</v>
+      </c>
+      <c r="D25" t="s">
+        <v>28</v>
+      </c>
+      <c r="E25" t="s">
+        <v>32</v>
+      </c>
+      <c r="F25" t="s">
+        <v>20</v>
+      </c>
+      <c r="G25" t="s">
+        <v>30</v>
+      </c>
+      <c r="H25" t="s">
+        <v>33</v>
+      </c>
+      <c r="I25" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>90</v>
+      </c>
+      <c r="B26" t="s">
+        <v>27</v>
+      </c>
+      <c r="C26" t="s">
+        <v>27</v>
+      </c>
+      <c r="D26" t="s">
+        <v>28</v>
+      </c>
+      <c r="E26" t="s">
+        <v>32</v>
+      </c>
+      <c r="F26" t="s">
+        <v>20</v>
+      </c>
+      <c r="G26" t="s">
+        <v>30</v>
+      </c>
+      <c r="I26" t="s">
+        <v>28</v>
+      </c>
+      <c r="J26" t="s">
+        <v>35</v>
+      </c>
+    </row>
   </sheetData>
   <conditionalFormatting sqref="A20">
     <cfRule type="duplicateValues" dxfId="1" priority="2"/>
@@ -1294,6 +1384,7 @@
     <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
   <ignoredErrors>
     <ignoredError sqref="A1:P15 B16:P16" numberStoredAsText="1"/>
   </ignoredErrors>

</xml_diff>